<commit_message>
Añade EAN 8410134017324 al cruce y personaliza texto de motivo Z2
Se añaden los 7 codigos SAP asociados al EAN 8410134017324 (linea
FRA/FR5 MANZ REL ANCHO). Ademas, el motivo literal de SAP "AC Falta
disponibilidad de la mercancia" ahora se muestra en Observaciones como
"Falta de disponibilidad informada".

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qh66VxXiVnYtXNz1pbfsEy
</commit_message>
<xml_diff>
--- a/data/cruce_ean_sap.xlsx
+++ b/data/cruce_ean_sap.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cruce_EAN_SAP" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cruce_EAN_SAP" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C604"/>
+  <dimension ref="A1:C611"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10684,6 +10684,125 @@
         </is>
       </c>
     </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>2007384</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>FRA MANZ REL ANCHO 22 12X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>2008772</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>FRA MANZ RELL ANCH 8X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>2010006</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>FRA MANZ REL ANCHO 22 12X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>2010107</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>FRA MANZ RELL ANCH 12X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>2010187</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>FRA MANZ RELL ANCH 12X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>2012574</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>FRA MANZ REL ANCHO 22 12X350 G</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>8410134017324</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>2012880</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>FR5 MANZ REL ANCHO 18 12X350 G</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nuevo texto para líneas sin incidencia y EAN 8410134026333 en el cruce
La observación de "sin incidencia" pasa a "No nos consta que esta
referencia haya presentado ninguna incidencia en este pedido." y el
resumen de la pantalla usa una etiqueta corta. Se añade el EAN
8410134026333 con el código SAP 2011483.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Qh66VxXiVnYtXNz1pbfsEy
</commit_message>
<xml_diff>
--- a/data/cruce_ean_sap.xlsx
+++ b/data/cruce_ean_sap.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C611"/>
+  <dimension ref="A1:C612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10803,6 +10803,19 @@
         </is>
       </c>
     </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>8410134026333</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>2011483</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>